<commit_message>
chore: update ESL schedules 2026-08-05
</commit_message>
<xml_diff>
--- a/output/esl_schedules_2026-08-05.xlsx
+++ b/output/esl_schedules_2026-08-05.xlsx
@@ -524,7 +524,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -908,7 +908,7 @@
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -956,7 +956,7 @@
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>29-Sep-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1100,7 +1100,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>29-Sep-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:06 UTC</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2356,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2548,7 +2548,7 @@
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2805,38 +2805,38 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>27-Sep-2026</t>
+          <t>28-Sep-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM / 026E6</t>
+          <t>EVER STEADY / 02639</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>12 days</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2848,43 +2848,43 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>EVER STEADY / 02639</t>
+          <t>KMT TBN / 02641</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>12 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2896,12 +2896,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2911,28 +2911,28 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>KMT TBN / 02641</t>
+          <t>BHUDTHI BHUM / 026E6</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3500,7 +3500,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3604,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3656,7 +3656,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3985,42 +3985,42 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>27-Sep-2026</t>
+          <t>28-Sep-2026</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>EVER STEADY</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02639</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>KHOR FAKKAN</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>20-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4032,47 +4032,47 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>EVER STEADY</t>
+          <t>KMT TBN</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>02639</t>
+          <t>02641</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4084,27 +4084,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>QINGDAO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>15-Oct-2026</t>
+          <t>02-Oct-2026</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>KMT TBN</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>02641</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4114,17 +4114,17 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>25-Oct-2026</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-08-05 04:20 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4816,7 @@
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5472,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>2026-08-05 04:21 UTC</t>
+          <t>2026-08-05 06:07 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update schedules 2026-08-05
</commit_message>
<xml_diff>
--- a/output/esl_schedules_2026-08-05.xlsx
+++ b/output/esl_schedules_2026-08-05.xlsx
@@ -524,7 +524,7 @@
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       <c r="I3" t="inlineStr"/>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -620,7 +620,7 @@
       <c r="I4" t="inlineStr"/>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -668,7 +668,7 @@
       <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
       <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>10-Sep-2026</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -887,12 +887,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>30-Sep-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM / 026E1</t>
+          <t>ESL NINGBO / 026E2</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -902,13 +902,13 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>20 days</t>
+          <t>17 days</t>
         </is>
       </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -925,7 +925,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>13-Sep-2026</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -935,12 +935,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>ESL NINGBO / 026E2</t>
+          <t>ESL NHAVA SHEVA / 026E3</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -950,13 +950,13 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>17 days</t>
+          <t>21 days</t>
         </is>
       </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1004,7 +1004,7 @@
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1100,7 +1100,7 @@
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1148,7 +1148,7 @@
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1200,7 +1200,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1356,7 +1356,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1460,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1581,7 +1581,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>10-Sep-2026</t>
+          <t>12-Sep-2026</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1591,12 +1591,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>026E1</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1606,17 +1606,17 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>30-Sep-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>21</t>
+          <t>18</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>14-Sep-2026</t>
+          <t>13-Sep-2026</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1643,12 +1643,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL NHAVA SHEVA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1658,17 +1658,17 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>22</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1720,7 +1720,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1772,7 +1772,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>04-Oct-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -1824,7 +1824,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>2026-08-05 06:06 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       <c r="I30" t="inlineStr"/>
       <c r="J30" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       <c r="I31" t="inlineStr"/>
       <c r="J31" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2020,7 +2020,7 @@
       <c r="I32" t="inlineStr"/>
       <c r="J32" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2068,7 +2068,7 @@
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2116,7 +2116,7 @@
       <c r="I34" t="inlineStr"/>
       <c r="J34" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       <c r="I35" t="inlineStr"/>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2212,7 +2212,7 @@
       <c r="I36" t="inlineStr"/>
       <c r="J36" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2260,7 +2260,7 @@
       <c r="I37" t="inlineStr"/>
       <c r="J37" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       <c r="I38" t="inlineStr"/>
       <c r="J38" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>02-Sep-2026</t>
+          <t>01-Sep-2026</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2335,7 +2335,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>25-Sep-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2356,7 +2356,7 @@
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2404,7 +2404,7 @@
       <c r="I40" t="inlineStr"/>
       <c r="J40" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2452,7 +2452,7 @@
       <c r="I41" t="inlineStr"/>
       <c r="J41" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>07-Sep-2026</t>
+          <t>10-Sep-2026</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2479,12 +2479,12 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>30-Sep-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM / 026E1</t>
+          <t>ESL NINGBO / 026E2</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2494,13 +2494,13 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>19 days</t>
         </is>
       </c>
       <c r="I42" t="inlineStr"/>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2517,7 +2517,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>12-Sep-2026</t>
+          <t>11-Sep-2026</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2527,12 +2527,12 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>ESL NINGBO / 026E2</t>
+          <t>ESL NHAVA SHEVA / 026E3</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2542,13 +2542,13 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>19 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I43" t="inlineStr"/>
       <c r="J43" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2596,7 +2596,7 @@
       <c r="I44" t="inlineStr"/>
       <c r="J44" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2644,7 +2644,7 @@
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2740,7 +2740,7 @@
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       <c r="I48" t="inlineStr"/>
       <c r="J48" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2805,38 +2805,38 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>27-Sep-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>EVER STEADY / 02639</t>
+          <t>BHUDTHI BHUM / 026E6</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>12 days</t>
+          <t>23 days</t>
         </is>
       </c>
       <c r="I49" t="inlineStr"/>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2848,43 +2848,43 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
           <t>PORT KLANG</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
-        <is>
-          <t>15-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>KMT TBN / 02641</t>
+          <t>EVER STEADY / 02639</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>EVGI</t>
+          <t>ECSX</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>16 days</t>
+          <t>12 days</t>
         </is>
       </c>
       <c r="I50" t="inlineStr"/>
       <c r="J50" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2896,12 +2896,12 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2911,28 +2911,28 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM / 026E6</t>
+          <t>KMT TBN / 02641</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>23 days</t>
+          <t>16 days</t>
         </is>
       </c>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,7 @@
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3084,7 +3084,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3136,7 +3136,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3240,7 +3240,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3292,7 +3292,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3344,7 +3344,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3396,7 +3396,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3465,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>02-Sep-2026</t>
+          <t>01-Sep-2026</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -3490,7 +3490,7 @@
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>25-Sep-2026</t>
+          <t>24-Sep-2026</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3552,7 +3552,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3604,7 +3604,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3621,7 +3621,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>07-Sep-2026</t>
+          <t>10-Sep-2026</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3631,12 +3631,12 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>KMTC DAMMAM</t>
+          <t>ESL NINGBO</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>026E1</t>
+          <t>026E2</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3646,17 +3646,17 @@
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>30-Sep-2026</t>
+          <t>29-Sep-2026</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>20</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3673,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>12-Sep-2026</t>
+          <t>11-Sep-2026</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3683,12 +3683,12 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>ESL NINGBO</t>
+          <t>ESL NHAVA SHEVA</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>026E2</t>
+          <t>026E3</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -3698,17 +3698,17 @@
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>01-Oct-2026</t>
+          <t>04-Oct-2026</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3812,7 +3812,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3864,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3916,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3968,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3985,42 +3985,42 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>28-Sep-2026</t>
+          <t>27-Sep-2026</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>ECSX</t>
+          <t>EGLX</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>EVER STEADY</t>
+          <t>BHUDTHI BHUM</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>02639</t>
+          <t>026E6</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>PORT KLANG</t>
+          <t>KHOR FAKKAN</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>10-Oct-2026</t>
+          <t>20-Oct-2026</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>24</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4032,47 +4032,47 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>QINGDAO</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>28-Sep-2026</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ECSX</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>EVER STEADY</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>02639</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
           <t>PORT KLANG</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>15-Oct-2026</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>EVGI</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>KMT TBN</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>02641</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>KHOR FAKKAN</t>
-        </is>
-      </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>31-Oct-2026</t>
+          <t>10-Oct-2026</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>13</t>
         </is>
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4084,27 +4084,27 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>QINGDAO</t>
+          <t>PORT KLANG</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>02-Oct-2026</t>
+          <t>15-Oct-2026</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>EGLX</t>
+          <t>EVGI</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>BHUDTHI BHUM</t>
+          <t>KMT TBN</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>026E6</t>
+          <t>02641</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -4114,17 +4114,17 @@
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>25-Oct-2026</t>
+          <t>31-Oct-2026</t>
         </is>
       </c>
       <c r="I74" t="inlineStr">
         <is>
-          <t>24</t>
+          <t>17</t>
         </is>
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4176,7 +4176,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4224,7 +4224,7 @@
       <c r="I76" t="inlineStr"/>
       <c r="J76" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       <c r="I77" t="inlineStr"/>
       <c r="J77" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4320,7 +4320,7 @@
       <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4368,7 +4368,7 @@
       <c r="I79" t="inlineStr"/>
       <c r="J79" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4420,7 +4420,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4472,7 +4472,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4524,7 +4524,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4624,7 +4624,7 @@
       <c r="I84" t="inlineStr"/>
       <c r="J84" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4672,7 +4672,7 @@
       <c r="I85" t="inlineStr"/>
       <c r="J85" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4720,7 +4720,7 @@
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       <c r="I87" t="inlineStr"/>
       <c r="J87" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4816,7 +4816,7 @@
       <c r="I88" t="inlineStr"/>
       <c r="J88" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4864,7 +4864,7 @@
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4912,7 +4912,7 @@
       <c r="I90" t="inlineStr"/>
       <c r="J90" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -4960,7 +4960,7 @@
       <c r="I91" t="inlineStr"/>
       <c r="J91" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5008,7 +5008,7 @@
       <c r="I92" t="inlineStr"/>
       <c r="J92" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5056,7 @@
       <c r="I93" t="inlineStr"/>
       <c r="J93" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5160,7 +5160,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5212,7 +5212,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5316,7 +5316,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5368,7 +5368,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5420,7 +5420,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5472,7 +5472,7 @@
       </c>
       <c r="J101" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       </c>
       <c r="J102" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="J103" t="inlineStr">
         <is>
-          <t>2026-08-05 06:07 UTC</t>
+          <t>2026-08-05 07:58 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>